<commit_message>
Add Murska Sobota project setup and analysis updates
</commit_message>
<xml_diff>
--- a/data/Murska_Sobota_2016-2024.xlsx
+++ b/data/Murska_Sobota_2016-2024.xlsx
@@ -5,18 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ijssi-my.sharepoint.com/personal/jan_gacnik_ijs_si/Documents/Jan 2023+/Voda izotopi Polona/Murska Sobota/Geologija_data_analysis/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ijssi-my.sharepoint.com/personal/jan_gacnik_ijs_si/Documents/Jan 2023+/Voda izotopi Polona/Murska Sobota/Data_analysis_MS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{D918F144-E6F6-422D-B54C-4A899681E75F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3223FFBE-2134-4B29-8905-1B56238A1F80}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{DDAB42A6-3E0F-4678-96B7-9C06406E4814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4A5068E-52BF-4C35-B206-455614A2FC7B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ESRI_MAPINFO_SHEET" sheetId="2" state="veryHidden" r:id="rId1"/>
     <sheet name="Data MS" sheetId="7" r:id="rId2"/>
+    <sheet name="Data all" sheetId="8" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Data all'!$A$1:$Q$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data MS'!$A$1:$AG$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2283" uniqueCount="158">
   <si>
     <t>Name</t>
   </si>
@@ -778,6 +780,15 @@
       </rPr>
       <t>H analysis</t>
     </r>
+  </si>
+  <si>
+    <t>Törökkoppány</t>
+  </si>
+  <si>
+    <t>Tamási</t>
+  </si>
+  <si>
+    <t>Koppány watershed</t>
   </si>
 </sst>
 </file>
@@ -1004,7 +1015,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1147,6 +1158,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2576,21 +2589,11 @@
       <c r="Z12" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="AA12" s="45">
-        <v>4.5</v>
-      </c>
-      <c r="AB12" s="27">
-        <v>0.6</v>
-      </c>
-      <c r="AC12" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="AD12" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="AE12" s="8" t="s">
-        <v>50</v>
-      </c>
+      <c r="AA12" s="45"/>
+      <c r="AB12" s="27"/>
+      <c r="AC12" s="9"/>
+      <c r="AD12" s="8"/>
+      <c r="AE12" s="8"/>
       <c r="AF12" s="15" t="s">
         <v>91</v>
       </c>
@@ -12176,4 +12179,2189 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{646F9698-2405-4D09-A201-C32B14251E82}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H87"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" style="4" customWidth="1"/>
+    <col min="4" max="5" width="7.44140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="7"/>
+    <col min="7" max="8" width="9.109375" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="50" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="18">
+        <v>2022</v>
+      </c>
+      <c r="C2" s="18">
+        <v>12</v>
+      </c>
+      <c r="D2" s="18">
+        <v>72.8</v>
+      </c>
+      <c r="E2" s="18">
+        <v>2.1</v>
+      </c>
+      <c r="F2" s="17">
+        <v>-13.91</v>
+      </c>
+      <c r="G2" s="17">
+        <v>-98.1</v>
+      </c>
+      <c r="H2" s="17">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C3" s="18">
+        <v>1</v>
+      </c>
+      <c r="D3" s="18">
+        <v>133.69999999999999</v>
+      </c>
+      <c r="E3" s="18">
+        <v>3.5</v>
+      </c>
+      <c r="F3" s="17">
+        <v>-14.5</v>
+      </c>
+      <c r="G3" s="17">
+        <v>-104.1</v>
+      </c>
+      <c r="H3" s="17">
+        <v>11.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C4" s="18">
+        <v>2</v>
+      </c>
+      <c r="D4" s="18">
+        <v>7</v>
+      </c>
+      <c r="E4" s="18">
+        <v>2.7</v>
+      </c>
+      <c r="F4" s="17">
+        <v>-10.34</v>
+      </c>
+      <c r="G4" s="17">
+        <v>-72.7</v>
+      </c>
+      <c r="H4" s="17">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C5" s="18">
+        <v>3</v>
+      </c>
+      <c r="D5" s="18">
+        <v>55.1</v>
+      </c>
+      <c r="E5" s="18">
+        <v>7.5</v>
+      </c>
+      <c r="F5" s="17">
+        <v>-10.93</v>
+      </c>
+      <c r="G5" s="17">
+        <v>-79.2</v>
+      </c>
+      <c r="H5" s="17">
+        <v>8.1999999999999993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C6" s="18">
+        <v>4</v>
+      </c>
+      <c r="D6" s="18">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="E6" s="18">
+        <v>9.5</v>
+      </c>
+      <c r="F6" s="17">
+        <v>-9.6300000000000008</v>
+      </c>
+      <c r="G6" s="17">
+        <v>-69</v>
+      </c>
+      <c r="H6" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C7" s="18">
+        <v>5</v>
+      </c>
+      <c r="D7" s="18">
+        <v>125.8</v>
+      </c>
+      <c r="E7" s="18">
+        <v>15.1</v>
+      </c>
+      <c r="F7" s="17">
+        <v>-7.39</v>
+      </c>
+      <c r="G7" s="17">
+        <v>-47.3</v>
+      </c>
+      <c r="H7" s="17">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C8" s="18">
+        <v>6</v>
+      </c>
+      <c r="D8" s="18">
+        <v>84.8</v>
+      </c>
+      <c r="E8" s="18">
+        <v>19.899999999999999</v>
+      </c>
+      <c r="F8" s="17">
+        <v>-6.68</v>
+      </c>
+      <c r="G8" s="17">
+        <v>-47.7</v>
+      </c>
+      <c r="H8" s="17">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C9" s="18">
+        <v>7</v>
+      </c>
+      <c r="D9" s="18">
+        <v>163.9</v>
+      </c>
+      <c r="E9" s="18">
+        <v>21.9</v>
+      </c>
+      <c r="F9" s="17">
+        <v>-4.7699999999999996</v>
+      </c>
+      <c r="G9" s="17">
+        <v>-30.3</v>
+      </c>
+      <c r="H9" s="17">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C10" s="18">
+        <v>8</v>
+      </c>
+      <c r="D10" s="18">
+        <v>136.80000000000001</v>
+      </c>
+      <c r="E10" s="18">
+        <v>20.8</v>
+      </c>
+      <c r="F10" s="17">
+        <v>-6.27</v>
+      </c>
+      <c r="G10" s="17">
+        <v>-38.799999999999997</v>
+      </c>
+      <c r="H10" s="17">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C11" s="18">
+        <v>9</v>
+      </c>
+      <c r="D11" s="18">
+        <v>31.9</v>
+      </c>
+      <c r="E11" s="18">
+        <v>18.3</v>
+      </c>
+      <c r="F11" s="17">
+        <v>-6.86</v>
+      </c>
+      <c r="G11" s="17">
+        <v>-49.8</v>
+      </c>
+      <c r="H11" s="17">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C12" s="18">
+        <v>10</v>
+      </c>
+      <c r="D12" s="18">
+        <v>54.5</v>
+      </c>
+      <c r="E12" s="18">
+        <v>14.3</v>
+      </c>
+      <c r="F12" s="17">
+        <v>-8.49</v>
+      </c>
+      <c r="G12" s="17">
+        <v>-60.5</v>
+      </c>
+      <c r="H12" s="17">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C13" s="18">
+        <v>11</v>
+      </c>
+      <c r="D13" s="18">
+        <v>82.3</v>
+      </c>
+      <c r="E13" s="18">
+        <v>5.8</v>
+      </c>
+      <c r="F13" s="17">
+        <v>-9.67</v>
+      </c>
+      <c r="G13" s="17">
+        <v>-65.900000000000006</v>
+      </c>
+      <c r="H13" s="17">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="27">
+        <v>2023</v>
+      </c>
+      <c r="C14" s="27">
+        <v>12</v>
+      </c>
+      <c r="D14" s="27">
+        <v>75.2</v>
+      </c>
+      <c r="E14" s="27">
+        <v>1.9</v>
+      </c>
+      <c r="F14" s="19">
+        <v>-15.15</v>
+      </c>
+      <c r="G14" s="19">
+        <v>-111.2</v>
+      </c>
+      <c r="H14" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C15" s="18">
+        <v>5</v>
+      </c>
+      <c r="D15" s="18">
+        <v>119.7</v>
+      </c>
+      <c r="E15" s="18">
+        <v>16.5</v>
+      </c>
+      <c r="F15" s="17">
+        <v>-5.9</v>
+      </c>
+      <c r="G15" s="17">
+        <v>-36.9</v>
+      </c>
+      <c r="H15" s="17">
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C16" s="18">
+        <v>6</v>
+      </c>
+      <c r="D16" s="18">
+        <v>74.3</v>
+      </c>
+      <c r="E16" s="18">
+        <v>21.3</v>
+      </c>
+      <c r="F16" s="17">
+        <v>-6.05</v>
+      </c>
+      <c r="G16" s="17">
+        <v>-41.8</v>
+      </c>
+      <c r="H16" s="17">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C17" s="18">
+        <v>8</v>
+      </c>
+      <c r="D17" s="18">
+        <v>51.4</v>
+      </c>
+      <c r="E17" s="18">
+        <v>23.5</v>
+      </c>
+      <c r="F17" s="17">
+        <v>-4.21</v>
+      </c>
+      <c r="G17" s="17">
+        <v>-28.6</v>
+      </c>
+      <c r="H17" s="17">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C18" s="18">
+        <v>9</v>
+      </c>
+      <c r="D18" s="18">
+        <v>164.3</v>
+      </c>
+      <c r="E18" s="18">
+        <v>16.5</v>
+      </c>
+      <c r="F18" s="17">
+        <v>-9.5399999999999991</v>
+      </c>
+      <c r="G18" s="17">
+        <v>-66.2</v>
+      </c>
+      <c r="H18" s="17">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C19" s="18">
+        <v>10</v>
+      </c>
+      <c r="D19" s="18">
+        <v>84.7</v>
+      </c>
+      <c r="E19" s="18">
+        <v>12.4</v>
+      </c>
+      <c r="F19" s="17">
+        <v>-10.32</v>
+      </c>
+      <c r="G19" s="17">
+        <v>-72</v>
+      </c>
+      <c r="H19" s="17">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C20" s="18">
+        <v>11</v>
+      </c>
+      <c r="D20" s="18">
+        <v>34.4</v>
+      </c>
+      <c r="E20" s="18">
+        <v>3.8</v>
+      </c>
+      <c r="F20" s="17">
+        <v>-13.38</v>
+      </c>
+      <c r="G20" s="17">
+        <v>-94.3</v>
+      </c>
+      <c r="H20" s="17">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C21" s="27">
+        <v>12</v>
+      </c>
+      <c r="D21" s="18">
+        <v>5</v>
+      </c>
+      <c r="E21" s="18">
+        <v>1.6</v>
+      </c>
+      <c r="F21" s="17">
+        <v>-13.19</v>
+      </c>
+      <c r="G21" s="17">
+        <v>-94.4</v>
+      </c>
+      <c r="H21" s="17">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B22" s="18">
+        <v>2022</v>
+      </c>
+      <c r="C22" s="18">
+        <v>12</v>
+      </c>
+      <c r="D22" s="41">
+        <v>75</v>
+      </c>
+      <c r="E22" s="55">
+        <v>2.9</v>
+      </c>
+      <c r="F22" s="17">
+        <v>-11.92</v>
+      </c>
+      <c r="G22" s="17">
+        <v>-84</v>
+      </c>
+      <c r="H22" s="17">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B23" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C23" s="18">
+        <v>1</v>
+      </c>
+      <c r="D23" s="41">
+        <v>109.9</v>
+      </c>
+      <c r="E23" s="55">
+        <v>4</v>
+      </c>
+      <c r="F23" s="17">
+        <v>-13.63</v>
+      </c>
+      <c r="G23" s="17">
+        <v>-95.5</v>
+      </c>
+      <c r="H23" s="17">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C24" s="18">
+        <v>2</v>
+      </c>
+      <c r="D24" s="41">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="E24" s="55">
+        <v>3.1</v>
+      </c>
+      <c r="F24" s="17">
+        <v>-15.51</v>
+      </c>
+      <c r="G24" s="17">
+        <v>-114.8</v>
+      </c>
+      <c r="H24" s="17">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B25" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C25" s="18">
+        <v>3</v>
+      </c>
+      <c r="D25" s="41">
+        <v>55.8</v>
+      </c>
+      <c r="E25" s="55">
+        <v>7.9</v>
+      </c>
+      <c r="F25" s="17">
+        <v>-8.66</v>
+      </c>
+      <c r="G25" s="17">
+        <v>-59.8</v>
+      </c>
+      <c r="H25" s="17">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B26" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C26" s="18">
+        <v>4</v>
+      </c>
+      <c r="D26" s="41">
+        <v>37.6</v>
+      </c>
+      <c r="E26" s="55">
+        <v>9.4</v>
+      </c>
+      <c r="F26" s="17">
+        <v>-7.52</v>
+      </c>
+      <c r="G26" s="17">
+        <v>-55.7</v>
+      </c>
+      <c r="H26" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C27" s="18">
+        <v>5</v>
+      </c>
+      <c r="D27" s="41">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="E27" s="55">
+        <v>15.4</v>
+      </c>
+      <c r="F27" s="17">
+        <v>-5</v>
+      </c>
+      <c r="G27" s="17">
+        <v>-28.2</v>
+      </c>
+      <c r="H27" s="17">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B28" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C28" s="18">
+        <v>6</v>
+      </c>
+      <c r="D28" s="41">
+        <v>93</v>
+      </c>
+      <c r="E28" s="55">
+        <v>19.7</v>
+      </c>
+      <c r="F28" s="17">
+        <v>-7.36</v>
+      </c>
+      <c r="G28" s="17">
+        <v>-55</v>
+      </c>
+      <c r="H28" s="17">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C29" s="18">
+        <v>7</v>
+      </c>
+      <c r="D29" s="41">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="E29" s="55">
+        <v>22.2</v>
+      </c>
+      <c r="F29" s="17">
+        <v>-3.65</v>
+      </c>
+      <c r="G29" s="17">
+        <v>-22.9</v>
+      </c>
+      <c r="H29" s="17">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C30" s="18">
+        <v>8</v>
+      </c>
+      <c r="D30" s="41">
+        <v>45.8</v>
+      </c>
+      <c r="E30" s="55">
+        <v>21.2</v>
+      </c>
+      <c r="F30" s="17"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C31" s="18">
+        <v>9</v>
+      </c>
+      <c r="D31" s="41">
+        <v>45.1</v>
+      </c>
+      <c r="E31" s="55">
+        <v>19</v>
+      </c>
+      <c r="F31" s="17">
+        <v>-7.33</v>
+      </c>
+      <c r="G31" s="17">
+        <v>-51.6</v>
+      </c>
+      <c r="H31" s="17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C32" s="18">
+        <v>10</v>
+      </c>
+      <c r="D32" s="41">
+        <v>48.1</v>
+      </c>
+      <c r="E32" s="55">
+        <v>14.6</v>
+      </c>
+      <c r="F32" s="17">
+        <v>-5.41</v>
+      </c>
+      <c r="G32" s="17">
+        <v>-41.5</v>
+      </c>
+      <c r="H32" s="17">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B33" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C33" s="18">
+        <v>11</v>
+      </c>
+      <c r="D33" s="41">
+        <v>104.8</v>
+      </c>
+      <c r="E33" s="55">
+        <v>6.8</v>
+      </c>
+      <c r="F33" s="17">
+        <v>-5.96</v>
+      </c>
+      <c r="G33" s="17">
+        <v>-38.5</v>
+      </c>
+      <c r="H33" s="17">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="27">
+        <v>2023</v>
+      </c>
+      <c r="C34" s="27">
+        <v>12</v>
+      </c>
+      <c r="D34" s="41">
+        <v>104.4</v>
+      </c>
+      <c r="E34" s="55">
+        <v>3.1</v>
+      </c>
+      <c r="F34" s="17">
+        <v>-9.6300000000000008</v>
+      </c>
+      <c r="G34" s="17">
+        <v>-71.7</v>
+      </c>
+      <c r="H34" s="17">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B35" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C35" s="18">
+        <v>5</v>
+      </c>
+      <c r="D35" s="41">
+        <v>53.4</v>
+      </c>
+      <c r="E35" s="55">
+        <v>17.7</v>
+      </c>
+      <c r="F35" s="17">
+        <v>-6.64</v>
+      </c>
+      <c r="G35" s="17">
+        <v>-49.3</v>
+      </c>
+      <c r="H35" s="17">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B36" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C36" s="18">
+        <v>6</v>
+      </c>
+      <c r="D36" s="41">
+        <v>97.9</v>
+      </c>
+      <c r="E36" s="55">
+        <v>21.5</v>
+      </c>
+      <c r="F36" s="17">
+        <v>-3.81</v>
+      </c>
+      <c r="G36" s="17">
+        <v>-23.3</v>
+      </c>
+      <c r="H36" s="17">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B37" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C37" s="18">
+        <v>8</v>
+      </c>
+      <c r="D37" s="41">
+        <v>9.1</v>
+      </c>
+      <c r="E37" s="55">
+        <v>24.9</v>
+      </c>
+      <c r="F37" s="17">
+        <v>-4.6399999999999997</v>
+      </c>
+      <c r="G37" s="17">
+        <v>-33.4</v>
+      </c>
+      <c r="H37" s="17">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B38" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C38" s="18">
+        <v>9</v>
+      </c>
+      <c r="D38" s="41">
+        <v>106</v>
+      </c>
+      <c r="E38" s="55">
+        <v>17.3</v>
+      </c>
+      <c r="F38" s="17">
+        <v>-10.23</v>
+      </c>
+      <c r="G38" s="17">
+        <v>-70.900000000000006</v>
+      </c>
+      <c r="H38" s="17">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B39" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C39" s="18">
+        <v>10</v>
+      </c>
+      <c r="D39" s="41">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="E39" s="55">
+        <v>11.9</v>
+      </c>
+      <c r="F39" s="17">
+        <v>-7.22</v>
+      </c>
+      <c r="G39" s="17">
+        <v>-54.7</v>
+      </c>
+      <c r="H39" s="17">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B40" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C40" s="18">
+        <v>11</v>
+      </c>
+      <c r="D40" s="41">
+        <v>42.5</v>
+      </c>
+      <c r="E40" s="55">
+        <v>4.2</v>
+      </c>
+      <c r="F40" s="17">
+        <v>-12.91</v>
+      </c>
+      <c r="G40" s="17">
+        <v>-94.8</v>
+      </c>
+      <c r="H40" s="17">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="54" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C41" s="27">
+        <v>12</v>
+      </c>
+      <c r="D41" s="41">
+        <v>25.3</v>
+      </c>
+      <c r="E41" s="55">
+        <v>2</v>
+      </c>
+      <c r="F41" s="17">
+        <v>-9.02</v>
+      </c>
+      <c r="G41" s="17">
+        <v>-70.599999999999994</v>
+      </c>
+      <c r="H41" s="17">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B42" s="18">
+        <v>2022</v>
+      </c>
+      <c r="C42" s="18">
+        <v>12</v>
+      </c>
+      <c r="D42" s="17">
+        <v>81.800000000000011</v>
+      </c>
+      <c r="E42" s="54"/>
+      <c r="F42" s="17"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C43" s="18">
+        <v>1</v>
+      </c>
+      <c r="D43" s="17">
+        <v>103.80000000000003</v>
+      </c>
+      <c r="E43" s="54"/>
+      <c r="F43" s="17"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B44" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C44" s="18">
+        <v>2</v>
+      </c>
+      <c r="D44" s="17">
+        <v>15.4</v>
+      </c>
+      <c r="E44" s="54"/>
+      <c r="F44" s="17">
+        <v>-15.03</v>
+      </c>
+      <c r="G44" s="17">
+        <v>-110.6</v>
+      </c>
+      <c r="H44" s="17">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B45" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C45" s="18">
+        <v>3</v>
+      </c>
+      <c r="D45" s="17">
+        <v>62.100000000000009</v>
+      </c>
+      <c r="E45" s="54"/>
+      <c r="F45" s="17">
+        <v>-8.2100000000000009</v>
+      </c>
+      <c r="G45" s="17">
+        <v>-56</v>
+      </c>
+      <c r="H45" s="17">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B46" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C46" s="18">
+        <v>4</v>
+      </c>
+      <c r="D46" s="17">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="E46" s="54"/>
+      <c r="F46" s="17">
+        <v>-7.83</v>
+      </c>
+      <c r="G46" s="17">
+        <v>-54.6</v>
+      </c>
+      <c r="H46" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B47" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C47" s="18">
+        <v>5</v>
+      </c>
+      <c r="D47" s="17">
+        <v>88.699999999999989</v>
+      </c>
+      <c r="E47" s="54"/>
+      <c r="F47" s="17">
+        <v>-7.71</v>
+      </c>
+      <c r="G47" s="17">
+        <v>-52.7</v>
+      </c>
+      <c r="H47" s="17">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B48" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C48" s="18">
+        <v>6</v>
+      </c>
+      <c r="D48" s="17">
+        <v>60.600000000000009</v>
+      </c>
+      <c r="E48" s="54"/>
+      <c r="F48" s="17">
+        <v>-6.26</v>
+      </c>
+      <c r="G48" s="17">
+        <v>-44.5</v>
+      </c>
+      <c r="H48" s="17">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B49" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C49" s="18">
+        <v>7</v>
+      </c>
+      <c r="D49" s="17">
+        <v>44.300000000000011</v>
+      </c>
+      <c r="E49" s="54"/>
+      <c r="F49" s="17">
+        <v>-5.01</v>
+      </c>
+      <c r="G49" s="17">
+        <v>-32.1</v>
+      </c>
+      <c r="H49" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B50" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C50" s="18">
+        <v>8</v>
+      </c>
+      <c r="D50" s="17">
+        <v>66</v>
+      </c>
+      <c r="E50" s="54"/>
+      <c r="F50" s="17">
+        <v>-4.5</v>
+      </c>
+      <c r="G50" s="17">
+        <v>-28</v>
+      </c>
+      <c r="H50" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B51" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C51" s="18">
+        <v>9</v>
+      </c>
+      <c r="D51" s="17">
+        <v>25.7</v>
+      </c>
+      <c r="E51" s="54"/>
+      <c r="F51" s="17">
+        <v>-6.8</v>
+      </c>
+      <c r="G51" s="17">
+        <v>-46.8</v>
+      </c>
+      <c r="H51" s="17">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B52" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C52" s="18">
+        <v>10</v>
+      </c>
+      <c r="D52" s="17">
+        <v>41.3</v>
+      </c>
+      <c r="E52" s="54"/>
+      <c r="F52" s="17">
+        <v>-7.88</v>
+      </c>
+      <c r="G52" s="17">
+        <v>-55.5</v>
+      </c>
+      <c r="H52" s="17">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B53" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C53" s="18">
+        <v>11</v>
+      </c>
+      <c r="D53" s="17">
+        <v>99.199999999999989</v>
+      </c>
+      <c r="E53" s="54"/>
+      <c r="F53" s="17">
+        <v>-8.93</v>
+      </c>
+      <c r="G53" s="17">
+        <v>-59.1</v>
+      </c>
+      <c r="H53" s="17">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" s="54" t="s">
+        <v>156</v>
+      </c>
+      <c r="B54" s="27">
+        <v>2023</v>
+      </c>
+      <c r="C54" s="27">
+        <v>12</v>
+      </c>
+      <c r="D54" s="17">
+        <v>114.20000000000002</v>
+      </c>
+      <c r="E54" s="54"/>
+      <c r="F54" s="17">
+        <v>-8.9700000000000006</v>
+      </c>
+      <c r="G54" s="17">
+        <v>-63.9</v>
+      </c>
+      <c r="H54" s="17">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B55" s="18">
+        <v>2022</v>
+      </c>
+      <c r="C55" s="18">
+        <v>12</v>
+      </c>
+      <c r="D55" s="41">
+        <v>75</v>
+      </c>
+      <c r="E55" s="55">
+        <v>2.9</v>
+      </c>
+      <c r="F55" s="17">
+        <v>-11.92</v>
+      </c>
+      <c r="G55" s="17">
+        <v>-84</v>
+      </c>
+      <c r="H55" s="17">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B56" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C56" s="18">
+        <v>1</v>
+      </c>
+      <c r="D56" s="41">
+        <v>109.9</v>
+      </c>
+      <c r="E56" s="55">
+        <v>4</v>
+      </c>
+      <c r="F56" s="17">
+        <v>-13.63</v>
+      </c>
+      <c r="G56" s="17">
+        <v>-95.5</v>
+      </c>
+      <c r="H56" s="17">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B57" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C57" s="18">
+        <v>2</v>
+      </c>
+      <c r="D57" s="41">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="E57" s="55">
+        <v>3.1</v>
+      </c>
+      <c r="F57" s="17">
+        <v>-15.51</v>
+      </c>
+      <c r="G57" s="17">
+        <v>-114.8</v>
+      </c>
+      <c r="H57" s="17">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B58" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C58" s="18">
+        <v>3</v>
+      </c>
+      <c r="D58" s="41">
+        <v>55.8</v>
+      </c>
+      <c r="E58" s="55">
+        <v>7.9</v>
+      </c>
+      <c r="F58" s="17">
+        <v>-8.66</v>
+      </c>
+      <c r="G58" s="17">
+        <v>-59.8</v>
+      </c>
+      <c r="H58" s="17">
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A59" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B59" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C59" s="18">
+        <v>4</v>
+      </c>
+      <c r="D59" s="41">
+        <v>37.6</v>
+      </c>
+      <c r="E59" s="55">
+        <v>9.4</v>
+      </c>
+      <c r="F59" s="17">
+        <v>-7.52</v>
+      </c>
+      <c r="G59" s="17">
+        <v>-55.7</v>
+      </c>
+      <c r="H59" s="17">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A60" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B60" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C60" s="18">
+        <v>5</v>
+      </c>
+      <c r="D60" s="41">
+        <v>76.599999999999994</v>
+      </c>
+      <c r="E60" s="55">
+        <v>15.4</v>
+      </c>
+      <c r="F60" s="17">
+        <v>-5</v>
+      </c>
+      <c r="G60" s="17">
+        <v>-28.2</v>
+      </c>
+      <c r="H60" s="17">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B61" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C61" s="18">
+        <v>6</v>
+      </c>
+      <c r="D61" s="41">
+        <v>93</v>
+      </c>
+      <c r="E61" s="55">
+        <v>19.7</v>
+      </c>
+      <c r="F61" s="17">
+        <v>-7.36</v>
+      </c>
+      <c r="G61" s="17">
+        <v>-55</v>
+      </c>
+      <c r="H61" s="17">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B62" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C62" s="18">
+        <v>7</v>
+      </c>
+      <c r="D62" s="41">
+        <v>74.900000000000006</v>
+      </c>
+      <c r="E62" s="55">
+        <v>22.2</v>
+      </c>
+      <c r="F62" s="17">
+        <v>-3.65</v>
+      </c>
+      <c r="G62" s="17">
+        <v>-22.9</v>
+      </c>
+      <c r="H62" s="17">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A63" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B63" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C63" s="18">
+        <v>8</v>
+      </c>
+      <c r="D63" s="41">
+        <v>45.8</v>
+      </c>
+      <c r="E63" s="55">
+        <v>21.2</v>
+      </c>
+      <c r="F63" s="17"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A64" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B64" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C64" s="18">
+        <v>9</v>
+      </c>
+      <c r="D64" s="41">
+        <v>45.1</v>
+      </c>
+      <c r="E64" s="55">
+        <v>19</v>
+      </c>
+      <c r="F64" s="17">
+        <v>-7.33</v>
+      </c>
+      <c r="G64" s="17">
+        <v>-51.6</v>
+      </c>
+      <c r="H64" s="17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B65" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C65" s="18">
+        <v>10</v>
+      </c>
+      <c r="D65" s="41">
+        <v>48.1</v>
+      </c>
+      <c r="E65" s="55">
+        <v>14.6</v>
+      </c>
+      <c r="F65" s="17">
+        <v>-5.41</v>
+      </c>
+      <c r="G65" s="17">
+        <v>-41.5</v>
+      </c>
+      <c r="H65" s="17">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A66" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B66" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C66" s="18">
+        <v>11</v>
+      </c>
+      <c r="D66" s="41">
+        <v>104.8</v>
+      </c>
+      <c r="E66" s="55">
+        <v>6.8</v>
+      </c>
+      <c r="F66" s="17">
+        <v>-5.96</v>
+      </c>
+      <c r="G66" s="17">
+        <v>-38.5</v>
+      </c>
+      <c r="H66" s="17">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A67" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B67" s="27">
+        <v>2023</v>
+      </c>
+      <c r="C67" s="27">
+        <v>12</v>
+      </c>
+      <c r="D67" s="41">
+        <v>104.4</v>
+      </c>
+      <c r="E67" s="55">
+        <v>3.1</v>
+      </c>
+      <c r="F67" s="17">
+        <v>-9.6300000000000008</v>
+      </c>
+      <c r="G67" s="17">
+        <v>-71.7</v>
+      </c>
+      <c r="H67" s="17">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A68" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B68" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C68" s="18">
+        <v>5</v>
+      </c>
+      <c r="D68" s="41">
+        <v>53.4</v>
+      </c>
+      <c r="E68" s="55">
+        <v>17.7</v>
+      </c>
+      <c r="F68" s="17">
+        <v>-6.64</v>
+      </c>
+      <c r="G68" s="17">
+        <v>-49.3</v>
+      </c>
+      <c r="H68" s="17">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B69" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C69" s="18">
+        <v>6</v>
+      </c>
+      <c r="D69" s="41">
+        <v>97.9</v>
+      </c>
+      <c r="E69" s="55">
+        <v>21.5</v>
+      </c>
+      <c r="F69" s="17">
+        <v>-3.81</v>
+      </c>
+      <c r="G69" s="17">
+        <v>-23.3</v>
+      </c>
+      <c r="H69" s="17">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A70" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B70" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C70" s="18">
+        <v>8</v>
+      </c>
+      <c r="D70" s="41">
+        <v>9.1</v>
+      </c>
+      <c r="E70" s="55">
+        <v>24.9</v>
+      </c>
+      <c r="F70" s="17">
+        <v>-4.6399999999999997</v>
+      </c>
+      <c r="G70" s="17">
+        <v>-33.4</v>
+      </c>
+      <c r="H70" s="17">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B71" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C71" s="18">
+        <v>9</v>
+      </c>
+      <c r="D71" s="41">
+        <v>106</v>
+      </c>
+      <c r="E71" s="55">
+        <v>17.3</v>
+      </c>
+      <c r="F71" s="17">
+        <v>-10.23</v>
+      </c>
+      <c r="G71" s="17">
+        <v>-70.900000000000006</v>
+      </c>
+      <c r="H71" s="17">
+        <v>10.9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A72" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B72" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C72" s="18">
+        <v>10</v>
+      </c>
+      <c r="D72" s="41">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="E72" s="55">
+        <v>11.9</v>
+      </c>
+      <c r="F72" s="17">
+        <v>-7.22</v>
+      </c>
+      <c r="G72" s="17">
+        <v>-54.7</v>
+      </c>
+      <c r="H72" s="17">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A73" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B73" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C73" s="18">
+        <v>11</v>
+      </c>
+      <c r="D73" s="41">
+        <v>42.5</v>
+      </c>
+      <c r="E73" s="55">
+        <v>4.2</v>
+      </c>
+      <c r="F73" s="17">
+        <v>-12.91</v>
+      </c>
+      <c r="G73" s="17">
+        <v>-94.8</v>
+      </c>
+      <c r="H73" s="17">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A74" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B74" s="18">
+        <v>2024</v>
+      </c>
+      <c r="C74" s="27">
+        <v>12</v>
+      </c>
+      <c r="D74" s="41">
+        <v>25.3</v>
+      </c>
+      <c r="E74" s="55">
+        <v>2</v>
+      </c>
+      <c r="F74" s="17">
+        <v>-9.02</v>
+      </c>
+      <c r="G74" s="17">
+        <v>-70.599999999999994</v>
+      </c>
+      <c r="H74" s="17">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B75" s="18">
+        <v>2022</v>
+      </c>
+      <c r="C75" s="18">
+        <v>12</v>
+      </c>
+      <c r="D75" s="17">
+        <v>81.800000000000011</v>
+      </c>
+      <c r="E75" s="54"/>
+      <c r="F75" s="17"/>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A76" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B76" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C76" s="18">
+        <v>1</v>
+      </c>
+      <c r="D76" s="17">
+        <v>103.80000000000003</v>
+      </c>
+      <c r="E76" s="54"/>
+      <c r="F76" s="17"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B77" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C77" s="18">
+        <v>2</v>
+      </c>
+      <c r="D77" s="17">
+        <v>15.4</v>
+      </c>
+      <c r="E77" s="54"/>
+      <c r="F77" s="17">
+        <v>-15.03</v>
+      </c>
+      <c r="G77" s="17">
+        <v>-110.6</v>
+      </c>
+      <c r="H77" s="17">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B78" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C78" s="18">
+        <v>3</v>
+      </c>
+      <c r="D78" s="17">
+        <v>62.100000000000009</v>
+      </c>
+      <c r="E78" s="54"/>
+      <c r="F78" s="17">
+        <v>-8.2100000000000009</v>
+      </c>
+      <c r="G78" s="17">
+        <v>-56</v>
+      </c>
+      <c r="H78" s="17">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A79" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B79" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C79" s="18">
+        <v>4</v>
+      </c>
+      <c r="D79" s="17">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="E79" s="54"/>
+      <c r="F79" s="17">
+        <v>-7.83</v>
+      </c>
+      <c r="G79" s="17">
+        <v>-54.6</v>
+      </c>
+      <c r="H79" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A80" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B80" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C80" s="18">
+        <v>5</v>
+      </c>
+      <c r="D80" s="17">
+        <v>88.699999999999989</v>
+      </c>
+      <c r="E80" s="54"/>
+      <c r="F80" s="17">
+        <v>-7.71</v>
+      </c>
+      <c r="G80" s="17">
+        <v>-52.7</v>
+      </c>
+      <c r="H80" s="17">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A81" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B81" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C81" s="18">
+        <v>6</v>
+      </c>
+      <c r="D81" s="17">
+        <v>60.600000000000009</v>
+      </c>
+      <c r="E81" s="54"/>
+      <c r="F81" s="17">
+        <v>-6.26</v>
+      </c>
+      <c r="G81" s="17">
+        <v>-44.5</v>
+      </c>
+      <c r="H81" s="17">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A82" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B82" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C82" s="18">
+        <v>7</v>
+      </c>
+      <c r="D82" s="17">
+        <v>44.300000000000011</v>
+      </c>
+      <c r="E82" s="54"/>
+      <c r="F82" s="17">
+        <v>-5.01</v>
+      </c>
+      <c r="G82" s="17">
+        <v>-32.1</v>
+      </c>
+      <c r="H82" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A83" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B83" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C83" s="18">
+        <v>8</v>
+      </c>
+      <c r="D83" s="17">
+        <v>66</v>
+      </c>
+      <c r="E83" s="54"/>
+      <c r="F83" s="17">
+        <v>-4.5</v>
+      </c>
+      <c r="G83" s="17">
+        <v>-28</v>
+      </c>
+      <c r="H83" s="17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A84" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B84" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C84" s="18">
+        <v>9</v>
+      </c>
+      <c r="D84" s="17">
+        <v>25.7</v>
+      </c>
+      <c r="E84" s="54"/>
+      <c r="F84" s="17">
+        <v>-6.8</v>
+      </c>
+      <c r="G84" s="17">
+        <v>-46.8</v>
+      </c>
+      <c r="H84" s="17">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A85" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B85" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C85" s="18">
+        <v>10</v>
+      </c>
+      <c r="D85" s="17">
+        <v>41.3</v>
+      </c>
+      <c r="E85" s="54"/>
+      <c r="F85" s="17">
+        <v>-7.88</v>
+      </c>
+      <c r="G85" s="17">
+        <v>-55.5</v>
+      </c>
+      <c r="H85" s="17">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A86" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B86" s="18">
+        <v>2023</v>
+      </c>
+      <c r="C86" s="18">
+        <v>11</v>
+      </c>
+      <c r="D86" s="17">
+        <v>99.199999999999989</v>
+      </c>
+      <c r="E86" s="54"/>
+      <c r="F86" s="17">
+        <v>-8.93</v>
+      </c>
+      <c r="G86" s="17">
+        <v>-59.1</v>
+      </c>
+      <c r="H86" s="17">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A87" s="54" t="s">
+        <v>157</v>
+      </c>
+      <c r="B87" s="27">
+        <v>2023</v>
+      </c>
+      <c r="C87" s="27">
+        <v>12</v>
+      </c>
+      <c r="D87" s="17">
+        <v>114.20000000000002</v>
+      </c>
+      <c r="E87" s="54"/>
+      <c r="F87" s="17">
+        <v>-8.9700000000000006</v>
+      </c>
+      <c r="G87" s="17">
+        <v>-63.9</v>
+      </c>
+      <c r="H87" s="17">
+        <v>7.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q116" xr:uid="{646F9698-2405-4D09-A201-C32B14251E82}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" scale="53" orientation="landscape" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>